<commit_message>
#5 Changes Update and Fresh Deliverables Generated.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/JLCPCB-BOM.xlsx
+++ b/Design_Files/BOM/JLCPCB-BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="117">
   <si>
     <t>Comment</t>
   </si>
@@ -45,6 +45,9 @@
     <t>4.7nF</t>
   </si>
   <si>
+    <t>20pF</t>
+  </si>
+  <si>
     <t>4.7uF</t>
   </si>
   <si>
@@ -114,7 +117,7 @@
     <t>CP2102N-A02-GQFN24R</t>
   </si>
   <si>
-    <t>CSTNE16M0VH3C000R0</t>
+    <t>X322516MLB4SI</t>
   </si>
   <si>
     <t>Designator</t>
@@ -141,6 +144,9 @@
     <t>C17</t>
   </si>
   <si>
+    <t>C21, C30</t>
+  </si>
+  <si>
     <t>C22, C23</t>
   </si>
   <si>
@@ -261,7 +267,7 @@
     <t>24-QFN (4x4)</t>
   </si>
   <si>
-    <t>SMD3213-3P</t>
+    <t>SMD3225-4P</t>
   </si>
   <si>
     <t>LCSC Part Number</t>
@@ -288,6 +294,9 @@
     <t>C107198</t>
   </si>
   <si>
+    <t>C107000</t>
+  </si>
+  <si>
     <t>C327025</t>
   </si>
   <si>
@@ -354,13 +363,13 @@
     <t>C969151</t>
   </si>
   <si>
-    <t>C882605</t>
+    <t>C13738</t>
+  </si>
+  <si>
+    <t>C5407657</t>
   </si>
   <si>
     <t>C2685197</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
 </sst>
 </file>
@@ -806,7 +815,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -820,13 +829,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -834,13 +843,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -848,13 +857,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -862,13 +871,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -876,13 +885,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -890,13 +899,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -904,13 +913,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -918,41 +927,41 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -960,13 +969,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -974,13 +983,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -988,13 +997,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1002,13 +1011,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1016,13 +1025,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>72</v>
+        <v>13</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1030,13 +1039,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1044,13 +1053,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>73</v>
+        <v>15</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1058,13 +1067,13 @@
         <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1072,13 +1081,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1086,13 +1095,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1100,13 +1109,13 @@
         <v>19</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1114,41 +1123,41 @@
         <v>20</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>101</v>
+      <c r="B23" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>102</v>
+      <c r="B24" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1156,13 +1165,13 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1170,13 +1179,13 @@
         <v>24</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1184,13 +1193,13 @@
         <v>25</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1198,13 +1207,13 @@
         <v>26</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1212,13 +1221,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1226,13 +1235,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1240,13 +1249,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1254,13 +1263,13 @@
         <v>30</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1268,13 +1277,27 @@
         <v>31</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>